<commit_message>
nit data correct central still has issue
</commit_message>
<xml_diff>
--- a/output_folder_2/NIRF NIT's_master_output.xlsx
+++ b/output_folder_2/NIRF NIT's_master_output.xlsx
@@ -648,7 +648,7 @@
     <col width="60" customWidth="1" min="218" max="218"/>
     <col width="57" customWidth="1" min="219" max="219"/>
     <col width="23" customWidth="1" min="220" max="220"/>
-    <col width="18" customWidth="1" min="221" max="221"/>
+    <col width="20" customWidth="1" min="221" max="221"/>
     <col width="48" customWidth="1" min="222" max="222"/>
     <col width="47" customWidth="1" min="223" max="223"/>
     <col width="50" customWidth="1" min="224" max="224"/>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="HM1" s="1" t="inlineStr">
         <is>
-          <t>Col_2:02-12-2016</t>
+          <t>Field_3:02-12-2016</t>
         </is>
       </c>
       <c r="HN1" s="1" t="inlineStr">

</xml_diff>